<commit_message>
Auto sales drop update: Sep_Target.xlsx
</commit_message>
<xml_diff>
--- a/Reports/Sep_Target.xlsx
+++ b/Reports/Sep_Target.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14856" windowHeight="10367"/>
+    <workbookView windowWidth="23040" windowHeight="10440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -107,7 +107,7 @@
     <t>RASHID MALL - JAZAN</t>
   </si>
   <si>
-    <t>208 MMS MDN</t>
+    <t>211 MMS MDN</t>
   </si>
   <si>
     <t>102 - Tala Mall(MMS)</t>
@@ -127,7 +127,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,13 +153,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -304,7 +297,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -350,12 +343,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,67 +682,70 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -770,73 +760,70 @@
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -870,7 +857,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1364,7 +1351,7 @@
         <v>180310</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" ht="22.8" spans="1:2">
       <c r="A23" s="9" t="s">
         <v>23</v>
       </c>

</xml_diff>